<commit_message>
Added fields Environment and Severity ti BugReport file
</commit_message>
<xml_diff>
--- a/Bug-Reports/Swag Labs_bug reports.xlsx
+++ b/Bug-Reports/Swag Labs_bug reports.xlsx
@@ -146,6 +146,21 @@
   </si>
   <si>
     <t>The error icons displayed next to the Username and Password fields are not clickable and do not clear the entered values.</t>
+  </si>
+  <si>
+    <t>Environment</t>
+  </si>
+  <si>
+    <t>Chrome - Version 147.0.7727.55</t>
+  </si>
+  <si>
+    <t>Steps to Reproduce</t>
+  </si>
+  <si>
+    <t>Severity</t>
+  </si>
+  <si>
+    <t>Medium</t>
   </si>
 </sst>
 </file>
@@ -234,7 +249,7 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>9</xdr:col>
+      <xdr:col>11</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>1</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
@@ -256,7 +271,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="9315450" y="361950"/>
+          <a:off x="12496800" y="190500"/>
           <a:ext cx="3295650" cy="2057400"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -577,10 +592,11 @@
     <col min="6" max="6" width="15.73828125" customWidth="1"/>
     <col min="7" max="7" width="16.94921875" customWidth="1"/>
     <col min="8" max="8" width="15.87109375" customWidth="1"/>
-    <col min="9" max="9" width="13.44921875" customWidth="1"/>
+    <col min="9" max="9" width="31.4765625" customWidth="1"/>
+    <col min="10" max="10" width="18.29296875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28.5">
+    <row r="1">
       <c r="A1" s="6" t="s">
         <v>13</v>
       </c>
@@ -600,7 +616,7 @@
         <v>3</v>
       </c>
       <c r="G1" s="6" t="s">
-        <v>4</v>
+        <v>38</v>
       </c>
       <c r="H1" s="7" t="s">
         <v>5</v>
@@ -608,7 +624,13 @@
       <c r="I1" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="J1" s="6" t="s">
+      <c r="J1" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="K1" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="L1" s="6" t="s">
         <v>7</v>
       </c>
     </row>
@@ -639,6 +661,12 @@
       </c>
       <c r="I2" s="1" t="s">
         <v>34</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="K2" t="s">
+        <v>40</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added new test casesand bug report to the files
</commit_message>
<xml_diff>
--- a/Bug-Reports/Swag Labs_bug reports.xlsx
+++ b/Bug-Reports/Swag Labs_bug reports.xlsx
@@ -9,11 +9,11 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="480" yWindow="75" windowWidth="18195" windowHeight="11820"/>
+    <workbookView xWindow="480" yWindow="75" windowWidth="18195" windowHeight="11820" activeTab="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
+    <sheet name="Login" sheetId="1" r:id="rId1"/>
+    <sheet name="Checkout" sheetId="4" r:id="rId7"/>
     <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="171027"/>
@@ -161,6 +161,61 @@
   </si>
   <si>
     <t>Medium</t>
+  </si>
+  <si>
+    <t>BR02</t>
+  </si>
+  <si>
+    <t>TS08</t>
+  </si>
+  <si>
+    <t>TC002</t>
+  </si>
+  <si>
+    <t>Checkout is Successful when the cart is Empty</t>
+  </si>
+  <si>
+    <t>Checkout is Successful when the Cart is Empty</t>
+  </si>
+  <si>
+    <t>The user can complete the checkout process successfully with an empty cart.
+The successful confirmation message appears.</t>
+  </si>
+  <si>
+    <t>1. The user is logged in and on the Cart page (https://www.saucedemo.com/cart.html)
+2. The shopping cart is empty</t>
+  </si>
+  <si>
+    <t>1. Click the 'Checkout' button
+2. Enter the valid data into the following fields: 
+- First Name
+- Last Name
+- Zip/Postal Code
+3. Click the 'Continue' button
+4. Click the 'Finish' button</t>
+  </si>
+  <si>
+    <t>Test Data</t>
+  </si>
+  <si>
+    <t>username: standard_user
+password: secret_sauce</t>
+  </si>
+  <si>
+    <t>username: standard_user
+password: secret_sauce
+First Name: Myname
+Last Name: Mylastname
+Zip/Postal Code: 123456</t>
+  </si>
+  <si>
+    <t>The user cannot complete the checkout process with an empty cart.
+The application keeps the user on the Cart page or prevents further checkout steps.</t>
+  </si>
+  <si>
+    <t>1. The checkout process is completed successfully.
+2. The confirmation message appears: 
+"Thank you for your order! Your order has been dispatched, and will arrive just as fast as the pony can get there!"</t>
   </si>
 </sst>
 </file>
@@ -634,53 +689,18 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" ht="163.5">
-      <c r="A2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B2" t="s">
-        <v>15</v>
-      </c>
-      <c r="C2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="G2" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="H2" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="I2" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="J2" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="K2" t="s">
-        <v>40</v>
-      </c>
+    <row r="2">
+      <c r="D2" s="1"/>
+      <c r="E2" s="1"/>
+      <c r="F2" s="1"/>
+      <c r="G2" s="1"/>
+      <c r="H2" s="1"/>
+      <c r="I2" s="1"/>
+      <c r="J2" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25" outlineLevelRow="0" outlineLevelCol="0"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
@@ -691,4 +711,105 @@
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25" outlineLevelRow="0" outlineLevelCol="0" defaultColWidth="8.609375"/>
+  <cols>
+    <col min="1" max="1" width="9.4140625" customWidth="1"/>
+    <col min="2" max="2" width="12.5078125" customWidth="1"/>
+    <col min="3" max="3" width="11.56640625" customWidth="1"/>
+    <col min="4" max="4" width="16.41015625" customWidth="1"/>
+    <col min="5" max="5" width="19.63671875" customWidth="1"/>
+    <col min="6" max="6" width="15.73828125" customWidth="1"/>
+    <col min="7" max="7" width="16.94921875" customWidth="1"/>
+    <col min="8" max="8" width="15.87109375" customWidth="1"/>
+    <col min="9" max="9" width="31.4765625" customWidth="1"/>
+    <col min="10" max="10" width="18.29296875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28.5">
+      <c r="A1" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="D1" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="E1" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="F1" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="G1" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="H1" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="I1" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="J1" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="K1" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="L1" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="M1" s="6" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" ht="163.5">
+      <c r="A2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" t="s">
+        <v>42</v>
+      </c>
+      <c r="C2" t="s">
+        <v>43</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="K2" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="L2" t="s">
+        <v>40</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>